<commit_message>
Updates to BIFUbC and PLANAbPiaSY
</commit_message>
<xml_diff>
--- a/InputData/land/PLANAbPiaSY/Potential Land Area Newly Affected by Pol in a Single Yr.xlsx
+++ b/InputData/land/PLANAbPiaSY/Potential Land Area Newly Affected by Pol in a Single Yr.xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28619"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29429"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/skorpius/My Drive/2024/FO local_EPS ICM/Diario/20250226_CATCHUP/land_CPL/PLANAbPiaSY/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2BA0548D-53DC-6D41-95F8-2DDE122A686A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="81" documentId="8_{2BA0548D-53DC-6D41-95F8-2DDE122A686A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8C235864-086F-4C92-BA72-94B12EEA6E90}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="33200" windowHeight="14600" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="33200" windowHeight="14600" firstSheet="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
     <sheet name="Potential Areas" sheetId="10" r:id="rId2"/>
-    <sheet name="Calculations &amp; Conversions" sheetId="11" r:id="rId3"/>
-    <sheet name="PLANAbPiaSY" sheetId="3" r:id="rId4"/>
+    <sheet name="CatOnBLU ICM data" sheetId="12" r:id="rId3"/>
+    <sheet name="Calculations &amp; Conversions" sheetId="11" r:id="rId4"/>
+    <sheet name="PLANAbPiaSY" sheetId="3" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="acres_per_million_hectares">#REF!</definedName>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="62">
   <si>
     <t>PLANAbPiaSY Potential Land Area Newly Affected by Policy in a Single Year</t>
   </si>
@@ -74,6 +75,94 @@
     <t xml:space="preserve">We considered Natural Protected Areas (ANP, in Spanish) as forest set-asides. </t>
   </si>
   <si>
+    <t>Climate Action Tool on Biodiversity &amp; Land Use</t>
+  </si>
+  <si>
+    <t>Resumen: Medidas de Mitigación</t>
+  </si>
+  <si>
+    <t>Costos por Implementación de Medidas de Mitigación</t>
+  </si>
+  <si>
+    <t>Id</t>
+  </si>
+  <si>
+    <t>Medida</t>
+  </si>
+  <si>
+    <t>Costo CAPEX
+[US2024/ha]</t>
+  </si>
+  <si>
+    <t>Costo OPEX
+[US2024/ha]</t>
+  </si>
+  <si>
+    <t>Años seguimiento</t>
+  </si>
+  <si>
+    <t>Costo Total Unitario
+[US2024/ha]</t>
+  </si>
+  <si>
+    <t>Costo Total
+[US2024/ha]</t>
+  </si>
+  <si>
+    <t>Meta</t>
+  </si>
+  <si>
+    <t>Unidad</t>
+  </si>
+  <si>
+    <t>Medida 1.1: Incrementar tierras forestales: regeneración natural asistida</t>
+  </si>
+  <si>
+    <t>Ha</t>
+  </si>
+  <si>
+    <t>Medida 1.1: Incrementar tierras forestales: enriquecimiento forestal</t>
+  </si>
+  <si>
+    <t>Medida 1.1: Incrementar tierras forestales: restauración activa</t>
+  </si>
+  <si>
+    <t>Medida 1.3: Fortalecer áreas de conservación</t>
+  </si>
+  <si>
+    <t>Medida 1.6: Fortalecer el manejo forestal sostenible</t>
+  </si>
+  <si>
+    <t>Medida 2.1: Incrementar superficie agrícola con agricultura de conservación</t>
+  </si>
+  <si>
+    <t>Medida 2.2: Restaurar la productividad de tierras agrícolas degradadas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Medida 2.3: Incrementar superficie agrícola con riego tecnificado </t>
+  </si>
+  <si>
+    <t>Medida 2.4: Incrementar superficie agrícola con sistemas agroforestales</t>
+  </si>
+  <si>
+    <t>Medida 3.1: Incrementar superficie de pastoreo mejorado</t>
+  </si>
+  <si>
+    <t>Medida 3.2: Incrementar superficie de pastoreo con sistemas silvopastoriles</t>
+  </si>
+  <si>
+    <t>km2</t>
+  </si>
+  <si>
+    <t>Ha/Km2</t>
+  </si>
+  <si>
+    <t>TOTAL HA</t>
+  </si>
+  <si>
+    <t>Total superficie República</t>
+  </si>
+  <si>
     <t>Potencial Técnico</t>
   </si>
   <si>
@@ -83,6 +172,9 @@
     <t>Forestry policy</t>
   </si>
   <si>
+    <t>CATONBLU 2060</t>
+  </si>
+  <si>
     <t>Set-asides</t>
   </si>
   <si>
@@ -114,6 +206,12 @@
   </si>
   <si>
     <t xml:space="preserve">Potencial Técnico </t>
+  </si>
+  <si>
+    <t>CATONBLU 2060 ICM DATA USED 2040 onwards, 2030-2040 period by linear ajustment</t>
+  </si>
+  <si>
+    <t>Original policy surface over</t>
   </si>
   <si>
     <t>years</t>
@@ -141,8 +239,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="174" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -176,7 +275,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -192,6 +291,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0" tint="-0.34998626667073579"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -251,7 +362,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -276,6 +387,15 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="4" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="1" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="1" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="174" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Comma" xfId="2" builtinId="3"/>
@@ -783,161 +903,715 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F4694B9B-AAE5-41B8-A6FE-9CA83ED3CBD8}">
+  <dimension ref="B2:L28"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="3" max="3" width="69.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="7.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:12">
+      <c r="C2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="2:12">
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="2:12">
+      <c r="B7" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" spans="2:12" ht="76.5">
+      <c r="B8" t="s">
+        <v>13</v>
+      </c>
+      <c r="C8" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="E8" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="F8" t="s">
+        <v>17</v>
+      </c>
+      <c r="G8" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="J8">
+        <v>2060</v>
+      </c>
+    </row>
+    <row r="9" spans="2:12" ht="60.75">
+      <c r="H9" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="I9" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="J9" t="s">
+        <v>20</v>
+      </c>
+      <c r="K9" t="s">
+        <v>21</v>
+      </c>
+      <c r="L9" s="14" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="10" spans="2:12">
+      <c r="B10">
+        <v>1</v>
+      </c>
+      <c r="C10" t="s">
+        <v>22</v>
+      </c>
+      <c r="D10">
+        <v>304</v>
+      </c>
+      <c r="E10">
+        <v>213</v>
+      </c>
+      <c r="F10">
+        <v>3</v>
+      </c>
+      <c r="G10">
+        <v>943</v>
+      </c>
+      <c r="H10" s="15">
+        <v>362889042.77999997</v>
+      </c>
+      <c r="I10" s="15">
+        <v>725778085.54999995</v>
+      </c>
+      <c r="J10" s="15">
+        <v>2693768.08</v>
+      </c>
+      <c r="K10" t="s">
+        <v>23</v>
+      </c>
+      <c r="L10" s="15">
+        <v>2540223299.4400001</v>
+      </c>
+    </row>
+    <row r="11" spans="2:12">
+      <c r="B11">
+        <v>2</v>
+      </c>
+      <c r="C11" t="s">
+        <v>24</v>
+      </c>
+      <c r="D11" s="15">
+        <v>1542</v>
+      </c>
+      <c r="E11">
+        <v>213</v>
+      </c>
+      <c r="F11">
+        <v>5</v>
+      </c>
+      <c r="G11" s="15">
+        <v>2607</v>
+      </c>
+      <c r="H11" s="15">
+        <v>2681576504.9200001</v>
+      </c>
+      <c r="I11" s="15">
+        <v>5363153009.8500004</v>
+      </c>
+      <c r="J11" s="15">
+        <v>7200243.7800000003</v>
+      </c>
+      <c r="K11" t="s">
+        <v>23</v>
+      </c>
+      <c r="L11" s="15">
+        <v>18771035534.459999</v>
+      </c>
+    </row>
+    <row r="12" spans="2:12">
+      <c r="B12">
+        <v>3</v>
+      </c>
+      <c r="C12" t="s">
+        <v>25</v>
+      </c>
+      <c r="D12" s="15">
+        <v>1048</v>
+      </c>
+      <c r="E12">
+        <v>213</v>
+      </c>
+      <c r="F12">
+        <v>5</v>
+      </c>
+      <c r="G12" s="15">
+        <v>2113</v>
+      </c>
+      <c r="H12" s="15">
+        <v>5253257103.3000002</v>
+      </c>
+      <c r="I12" s="15">
+        <v>10506514206.59</v>
+      </c>
+      <c r="J12" s="15">
+        <v>17403123.390000001</v>
+      </c>
+      <c r="K12" t="s">
+        <v>23</v>
+      </c>
+      <c r="L12" s="15">
+        <v>36772799723.07</v>
+      </c>
+    </row>
+    <row r="13" spans="2:12">
+      <c r="B13">
+        <v>4</v>
+      </c>
+      <c r="C13" t="s">
+        <v>26</v>
+      </c>
+      <c r="E13">
+        <v>14.49</v>
+      </c>
+      <c r="F13">
+        <v>35</v>
+      </c>
+      <c r="G13">
+        <v>507.21</v>
+      </c>
+      <c r="H13" s="15">
+        <v>12374814618.59</v>
+      </c>
+      <c r="I13" s="15">
+        <v>12374814618.59</v>
+      </c>
+      <c r="J13" s="15">
+        <v>24397601.129999999</v>
+      </c>
+      <c r="K13" t="s">
+        <v>23</v>
+      </c>
+      <c r="L13" s="15">
+        <v>12374814618.59</v>
+      </c>
+    </row>
+    <row r="14" spans="2:12">
+      <c r="B14">
+        <v>5</v>
+      </c>
+      <c r="C14" t="s">
+        <v>27</v>
+      </c>
+      <c r="E14">
+        <v>460.01</v>
+      </c>
+      <c r="F14">
+        <v>25</v>
+      </c>
+      <c r="G14" s="15">
+        <v>11500.25</v>
+      </c>
+      <c r="H14" s="15">
+        <v>13866015714.290001</v>
+      </c>
+      <c r="I14" s="15">
+        <v>27732031428.57</v>
+      </c>
+      <c r="J14" s="15">
+        <v>8440000</v>
+      </c>
+      <c r="K14" t="s">
+        <v>23</v>
+      </c>
+      <c r="L14" s="15">
+        <v>97062110000</v>
+      </c>
+    </row>
+    <row r="15" spans="2:12">
+      <c r="B15">
+        <v>6</v>
+      </c>
+      <c r="C15" t="s">
+        <v>28</v>
+      </c>
+      <c r="E15" s="15">
+        <v>2448.35</v>
+      </c>
+      <c r="F15">
+        <v>3</v>
+      </c>
+      <c r="G15" s="15">
+        <v>7345.05</v>
+      </c>
+      <c r="H15" s="15">
+        <v>3559312481.0500002</v>
+      </c>
+      <c r="I15" s="15">
+        <v>7118624962.1000004</v>
+      </c>
+      <c r="J15" s="15">
+        <v>3392105.89</v>
+      </c>
+      <c r="K15" t="s">
+        <v>23</v>
+      </c>
+      <c r="L15" s="15">
+        <v>24915187367.34</v>
+      </c>
+    </row>
+    <row r="16" spans="2:12">
+      <c r="B16">
+        <v>7</v>
+      </c>
+      <c r="C16" t="s">
+        <v>29</v>
+      </c>
+      <c r="E16" s="15">
+        <v>2833.59</v>
+      </c>
+      <c r="F16">
+        <v>3</v>
+      </c>
+      <c r="G16" s="15">
+        <v>8500.77</v>
+      </c>
+      <c r="H16" s="15">
+        <v>1619367150.9000001</v>
+      </c>
+      <c r="I16" s="15">
+        <v>3238734301.79</v>
+      </c>
+      <c r="J16" s="15">
+        <v>1333475.68</v>
+      </c>
+      <c r="K16" t="s">
+        <v>23</v>
+      </c>
+      <c r="L16" s="15">
+        <v>11335570056.27</v>
+      </c>
+    </row>
+    <row r="17" spans="2:12">
+      <c r="B17">
+        <v>8</v>
+      </c>
+      <c r="C17" t="s">
+        <v>30</v>
+      </c>
+      <c r="D17" s="15">
+        <v>9236.49</v>
+      </c>
+      <c r="E17" s="15">
+        <v>2349.84</v>
+      </c>
+      <c r="F17">
+        <v>3</v>
+      </c>
+      <c r="G17" s="15">
+        <v>16286</v>
+      </c>
+      <c r="H17" s="15">
+        <v>3081345121.0999999</v>
+      </c>
+      <c r="I17" s="15">
+        <v>6162690242.21</v>
+      </c>
+      <c r="J17" s="15">
+        <v>1324414.58</v>
+      </c>
+      <c r="K17" t="s">
+        <v>23</v>
+      </c>
+      <c r="L17" s="15">
+        <v>21569415847.720001</v>
+      </c>
+    </row>
+    <row r="18" spans="2:12">
+      <c r="B18">
+        <v>9</v>
+      </c>
+      <c r="C18" t="s">
+        <v>31</v>
+      </c>
+      <c r="D18" s="15">
+        <v>4193.09</v>
+      </c>
+      <c r="E18">
+        <v>937.98</v>
+      </c>
+      <c r="F18">
+        <v>4</v>
+      </c>
+      <c r="G18" s="15">
+        <v>7945</v>
+      </c>
+      <c r="H18" s="15">
+        <v>7410807710</v>
+      </c>
+      <c r="I18" s="15">
+        <v>14821615420</v>
+      </c>
+      <c r="J18" s="15">
+        <v>6529346</v>
+      </c>
+      <c r="K18" t="s">
+        <v>23</v>
+      </c>
+      <c r="L18" s="15">
+        <v>51875653970</v>
+      </c>
+    </row>
+    <row r="19" spans="2:12">
+      <c r="B19">
+        <v>10</v>
+      </c>
+      <c r="C19" t="s">
+        <v>32</v>
+      </c>
+      <c r="D19" s="15">
+        <v>3128.67</v>
+      </c>
+      <c r="E19" s="15">
+        <v>1199.28</v>
+      </c>
+      <c r="F19">
+        <v>3</v>
+      </c>
+      <c r="G19" s="15">
+        <v>6726.5</v>
+      </c>
+      <c r="H19" s="15">
+        <v>8293774500</v>
+      </c>
+      <c r="I19" s="15">
+        <v>16587549000</v>
+      </c>
+      <c r="J19" s="15">
+        <v>8631000</v>
+      </c>
+      <c r="K19" t="s">
+        <v>23</v>
+      </c>
+      <c r="L19" s="15">
+        <v>58056421500</v>
+      </c>
+    </row>
+    <row r="20" spans="2:12">
+      <c r="B20">
+        <v>11</v>
+      </c>
+      <c r="C20" t="s">
+        <v>33</v>
+      </c>
+      <c r="D20" s="15">
+        <v>3003.18</v>
+      </c>
+      <c r="E20">
+        <v>671.8</v>
+      </c>
+      <c r="F20">
+        <v>4</v>
+      </c>
+      <c r="G20" s="15">
+        <v>5690.38</v>
+      </c>
+      <c r="H20" s="15">
+        <v>3508119270</v>
+      </c>
+      <c r="I20" s="15">
+        <v>7016238540</v>
+      </c>
+      <c r="J20" s="15">
+        <v>4315500</v>
+      </c>
+      <c r="K20" t="s">
+        <v>23</v>
+      </c>
+      <c r="L20" s="15">
+        <v>24556834890</v>
+      </c>
+    </row>
+    <row r="22" spans="2:12">
+      <c r="H22" s="15">
+        <v>3044465547.6999998</v>
+      </c>
+      <c r="I22" s="15">
+        <v>6088931095.3999996</v>
+      </c>
+    </row>
+    <row r="25" spans="2:12">
+      <c r="G25" t="s">
+        <v>34</v>
+      </c>
+      <c r="H25" t="s">
+        <v>35</v>
+      </c>
+      <c r="I25" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="J25" s="17">
+        <v>85660578.530000001</v>
+      </c>
+      <c r="K25" s="16" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="26" spans="2:12">
+      <c r="G26">
+        <v>1964375</v>
+      </c>
+      <c r="H26">
+        <v>100</v>
+      </c>
+      <c r="I26" t="s">
+        <v>37</v>
+      </c>
+      <c r="J26" s="15">
+        <v>196437500</v>
+      </c>
+    </row>
+    <row r="28" spans="2:12">
+      <c r="J28">
+        <v>0.436070397</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A2:G15"/>
+  <dimension ref="A2:H20"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="21" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="25.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.85546875" customWidth="1"/>
+    <col min="4" max="4" width="16.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:7" ht="29.25" customHeight="1">
+    <row r="2" spans="1:8" ht="29.25" customHeight="1">
       <c r="A2" s="12" t="s">
-        <v>10</v>
+        <v>38</v>
       </c>
       <c r="B2" s="13"/>
       <c r="C2" s="11"/>
-    </row>
-    <row r="3" spans="1:7">
+      <c r="D2">
+        <f>'CatOnBLU ICM data'!J25/1000000</f>
+        <v>85.660578529999995</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
       <c r="A3" s="10" t="s">
-        <v>11</v>
+        <v>39</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>12</v>
+        <v>40</v>
       </c>
       <c r="C3" s="10">
         <v>2030</v>
       </c>
-    </row>
-    <row r="4" spans="1:7">
+      <c r="D3" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
       <c r="A4" s="8" t="s">
-        <v>13</v>
+        <v>42</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>14</v>
+        <v>43</v>
       </c>
       <c r="C4" s="8">
         <v>6</v>
       </c>
-    </row>
-    <row r="5" spans="1:7">
+      <c r="D4" s="15">
+        <f>'CatOnBLU ICM data'!J13/1000000</f>
+        <v>24.397601129999998</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
       <c r="A5" s="8" t="s">
-        <v>15</v>
+        <v>44</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>16</v>
+        <v>45</v>
       </c>
       <c r="C5" s="8">
         <v>4.2</v>
       </c>
-    </row>
-    <row r="6" spans="1:7">
+      <c r="D5">
+        <f>('CatOnBLU ICM data'!J10+'CatOnBLU ICM data'!J11+'CatOnBLU ICM data'!J12)/1000000</f>
+        <v>27.29713525</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
       <c r="A6" s="8" t="s">
-        <v>17</v>
+        <v>46</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>18</v>
+        <v>47</v>
       </c>
       <c r="C6" s="8">
         <v>18.7</v>
       </c>
-    </row>
-    <row r="7" spans="1:7">
+      <c r="D6" s="15">
+        <f>'CatOnBLU ICM data'!J14/1000000</f>
+        <v>8.44</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8">
       <c r="A7" s="8" t="s">
-        <v>17</v>
+        <v>46</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>19</v>
+        <v>48</v>
       </c>
       <c r="C7" s="8">
         <v>1.9</v>
       </c>
-      <c r="E7" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="F7" s="10"/>
-    </row>
-    <row r="8" spans="1:7">
-      <c r="E8" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="F8" s="8">
+      <c r="D7">
+        <f>SUM('CatOnBLU ICM data'!J15:J20)/1000000</f>
+        <v>25.525842149999999</v>
+      </c>
+      <c r="F7" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="G7" s="10"/>
+    </row>
+    <row r="8" spans="1:8">
+      <c r="F8" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="G8" s="8">
         <v>2.4700000000000002</v>
       </c>
-      <c r="G8" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7">
+      <c r="H8" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8">
       <c r="A10" s="12" t="s">
-        <v>23</v>
+        <v>52</v>
       </c>
       <c r="B10" s="13"/>
       <c r="C10" s="11"/>
-      <c r="E10" s="8">
-        <v>30</v>
-      </c>
-      <c r="F10" s="9" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7">
+    </row>
+    <row r="11" spans="1:8">
       <c r="A11" s="10" t="s">
-        <v>11</v>
+        <v>39</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>12</v>
+        <v>40</v>
       </c>
       <c r="C11" s="10">
         <v>2030</v>
       </c>
-    </row>
-    <row r="12" spans="1:7">
+      <c r="D11" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8">
       <c r="A12" s="8" t="s">
-        <v>13</v>
+        <v>42</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="C12" s="8">
-        <f>C4*$F$8*1000000</f>
+        <v>43</v>
+      </c>
+      <c r="C12" s="20">
+        <f>C4*$G$8*1000000</f>
         <v>14820000</v>
       </c>
-    </row>
-    <row r="13" spans="1:7">
+      <c r="D12" s="20">
+        <f>D4*$G$8*1000000</f>
+        <v>60262074.791099995</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8">
       <c r="A13" s="8" t="s">
-        <v>15</v>
+        <v>44</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="C13" s="8">
-        <f>C5*$F$8*1000000</f>
+        <v>45</v>
+      </c>
+      <c r="C13" s="20">
+        <f>C5*$G$8*1000000</f>
         <v>10374000</v>
       </c>
-    </row>
-    <row r="14" spans="1:7">
+      <c r="D13" s="20">
+        <f>D5*$G$8*1000000</f>
+        <v>67423924.06750001</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8">
       <c r="A14" s="8" t="s">
-        <v>17</v>
+        <v>46</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="C14" s="8">
-        <f>C6*$F$8*1000000</f>
+        <v>47</v>
+      </c>
+      <c r="C14" s="20">
+        <f>C6*$G$8*1000000</f>
         <v>46189000</v>
       </c>
-    </row>
-    <row r="15" spans="1:7">
+      <c r="D14" s="20">
+        <f>D6*$G$8*1000000</f>
+        <v>20846800</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8">
       <c r="A15" s="8" t="s">
-        <v>17</v>
+        <v>46</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="C15" s="8">
-        <f>C7*$F$8*1000000</f>
+        <v>48</v>
+      </c>
+      <c r="C15" s="20">
+        <f>C7*$G$8*1000000</f>
         <v>4693000.0000000009</v>
+      </c>
+      <c r="D15" s="20">
+        <f>D7*$G$8*1000000</f>
+        <v>63048830.1105</v>
+      </c>
+    </row>
+    <row r="17" spans="4:6">
+      <c r="D17" s="16" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="19" spans="4:6">
+      <c r="D19" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="E19" s="8">
+        <v>20</v>
+      </c>
+      <c r="F19" s="9" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="20" spans="4:6">
+      <c r="D20" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="E20" s="8">
+        <v>20</v>
+      </c>
+      <c r="F20" s="9" t="s">
+        <v>55</v>
       </c>
     </row>
   </sheetData>
@@ -950,7 +1624,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr>
     <tabColor theme="3"/>
@@ -1131,682 +1805,682 @@
     </row>
     <row r="2" spans="1:56">
       <c r="A2" t="s">
-        <v>25</v>
+        <v>56</v>
       </c>
       <c r="B2" s="3">
-        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$10</f>
-        <v>494000</v>
+        <f>'Calculations &amp; Conversions'!$C12/'Calculations &amp; Conversions'!$E$19</f>
+        <v>741000</v>
       </c>
       <c r="C2" s="3">
-        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$10</f>
-        <v>494000</v>
+        <f>'Calculations &amp; Conversions'!$C12/'Calculations &amp; Conversions'!$E$19</f>
+        <v>741000</v>
       </c>
       <c r="D2" s="3">
-        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$10</f>
-        <v>494000</v>
+        <f>'Calculations &amp; Conversions'!$C12/'Calculations &amp; Conversions'!$E$19</f>
+        <v>741000</v>
       </c>
       <c r="E2" s="3">
-        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$10</f>
-        <v>494000</v>
+        <f>'Calculations &amp; Conversions'!$C12/'Calculations &amp; Conversions'!$E$19</f>
+        <v>741000</v>
       </c>
       <c r="F2" s="3">
-        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$10</f>
-        <v>494000</v>
+        <f>'Calculations &amp; Conversions'!$C12/'Calculations &amp; Conversions'!$E$19</f>
+        <v>741000</v>
       </c>
       <c r="G2" s="3">
-        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$10</f>
-        <v>494000</v>
+        <f>'Calculations &amp; Conversions'!$C12/'Calculations &amp; Conversions'!$E$19</f>
+        <v>741000</v>
       </c>
       <c r="H2" s="3">
-        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$10</f>
-        <v>494000</v>
+        <f>'Calculations &amp; Conversions'!$C12/'Calculations &amp; Conversions'!$E$19</f>
+        <v>741000</v>
       </c>
       <c r="I2" s="3">
-        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$10</f>
-        <v>494000</v>
+        <f>'Calculations &amp; Conversions'!$C12/'Calculations &amp; Conversions'!$E$19</f>
+        <v>741000</v>
       </c>
       <c r="J2" s="3">
-        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$10</f>
-        <v>494000</v>
+        <f>'Calculations &amp; Conversions'!$C12/'Calculations &amp; Conversions'!$E$19</f>
+        <v>741000</v>
       </c>
       <c r="K2" s="3">
-        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$10</f>
-        <v>494000</v>
+        <f>'Calculations &amp; Conversions'!$C12/'Calculations &amp; Conversions'!$E$19</f>
+        <v>741000</v>
       </c>
       <c r="L2" s="3">
-        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$10</f>
-        <v>494000</v>
+        <f>'Calculations &amp; Conversions'!$C12/'Calculations &amp; Conversions'!$E$19</f>
+        <v>741000</v>
       </c>
       <c r="M2" s="3">
-        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$10</f>
-        <v>494000</v>
+        <f>'Calculations &amp; Conversions'!$C12/'Calculations &amp; Conversions'!$E$19</f>
+        <v>741000</v>
       </c>
       <c r="N2" s="3">
-        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$10</f>
-        <v>494000</v>
+        <f>'Calculations &amp; Conversions'!$C12/'Calculations &amp; Conversions'!$E$19</f>
+        <v>741000</v>
       </c>
       <c r="O2" s="3">
-        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$10</f>
-        <v>494000</v>
+        <f>'Calculations &amp; Conversions'!$C12/'Calculations &amp; Conversions'!$E$19</f>
+        <v>741000</v>
       </c>
       <c r="P2" s="3">
-        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$10</f>
-        <v>494000</v>
-      </c>
-      <c r="Q2" s="3">
-        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$10</f>
-        <v>494000</v>
-      </c>
-      <c r="R2" s="3">
-        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$10</f>
-        <v>494000</v>
-      </c>
-      <c r="S2" s="3">
-        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$10</f>
-        <v>494000</v>
-      </c>
-      <c r="T2" s="3">
-        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$10</f>
-        <v>494000</v>
-      </c>
-      <c r="U2" s="3">
-        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$10</f>
-        <v>494000</v>
-      </c>
-      <c r="V2" s="3">
-        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$10</f>
-        <v>494000</v>
-      </c>
-      <c r="W2" s="3">
-        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$10</f>
-        <v>494000</v>
-      </c>
-      <c r="X2" s="3">
-        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$10</f>
-        <v>494000</v>
-      </c>
-      <c r="Y2" s="3">
-        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$10</f>
-        <v>494000</v>
-      </c>
-      <c r="Z2" s="3">
-        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$10</f>
-        <v>494000</v>
-      </c>
-      <c r="AA2" s="3">
-        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$10</f>
-        <v>494000</v>
-      </c>
-      <c r="AB2" s="3">
-        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$10</f>
-        <v>494000</v>
-      </c>
-      <c r="AC2" s="3">
-        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$10</f>
-        <v>494000</v>
-      </c>
-      <c r="AD2" s="3">
-        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$10</f>
-        <v>494000</v>
-      </c>
-      <c r="AE2" s="3">
-        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$10</f>
-        <v>494000</v>
-      </c>
-      <c r="AF2" s="3">
-        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$10</f>
-        <v>494000</v>
-      </c>
-      <c r="AG2" s="3">
-        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$10</f>
-        <v>494000</v>
-      </c>
-      <c r="AH2" s="3">
-        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$10</f>
-        <v>494000</v>
-      </c>
-      <c r="AI2" s="3">
-        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$10</f>
-        <v>494000</v>
-      </c>
-      <c r="AJ2" s="3">
-        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$10</f>
-        <v>494000</v>
-      </c>
-      <c r="AK2" s="3">
-        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$10</f>
-        <v>494000</v>
-      </c>
-      <c r="AL2" s="3">
-        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$10</f>
-        <v>494000</v>
-      </c>
-      <c r="AM2" s="3">
-        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$10</f>
-        <v>494000</v>
-      </c>
-      <c r="AN2" s="3">
-        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$10</f>
-        <v>494000</v>
-      </c>
-      <c r="AO2" s="3">
-        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$10</f>
-        <v>494000</v>
-      </c>
-      <c r="AP2" s="3">
-        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$10</f>
-        <v>494000</v>
-      </c>
-      <c r="AQ2" s="3">
-        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$10</f>
-        <v>494000</v>
-      </c>
-      <c r="AR2" s="3">
-        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$10</f>
-        <v>494000</v>
-      </c>
-      <c r="AS2" s="3">
-        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$10</f>
-        <v>494000</v>
-      </c>
-      <c r="AT2" s="3">
-        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$10</f>
-        <v>494000</v>
-      </c>
-      <c r="AU2" s="3">
-        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$10</f>
-        <v>494000</v>
-      </c>
-      <c r="AV2" s="3">
-        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$10</f>
-        <v>494000</v>
-      </c>
-      <c r="AW2" s="3">
-        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$10</f>
-        <v>494000</v>
-      </c>
-      <c r="AX2" s="3">
-        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$10</f>
-        <v>494000</v>
-      </c>
-      <c r="AY2" s="3">
-        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$10</f>
-        <v>494000</v>
-      </c>
-      <c r="AZ2" s="3">
-        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$10</f>
-        <v>494000</v>
-      </c>
-      <c r="BA2" s="3">
-        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$10</f>
-        <v>494000</v>
-      </c>
-      <c r="BB2" s="3">
-        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$10</f>
-        <v>494000</v>
-      </c>
-      <c r="BC2" s="3">
-        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$10</f>
-        <v>494000</v>
-      </c>
-      <c r="BD2" s="3">
-        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$10</f>
-        <v>494000</v>
+        <f>'Calculations &amp; Conversions'!$C12/'Calculations &amp; Conversions'!$E$19</f>
+        <v>741000</v>
+      </c>
+      <c r="Q2" s="18">
+        <f>(Z2-P2)/(Z$1-P$1)*(Q$1-$P$1)+$P2</f>
+        <v>741000</v>
+      </c>
+      <c r="R2" s="18">
+        <f t="shared" ref="R2:Y2" si="0">(AA2-Q2)/(AA$1-Q$1)*(R$1-$P$1)+$P2</f>
+        <v>741000</v>
+      </c>
+      <c r="S2" s="18">
+        <f t="shared" si="0"/>
+        <v>741000</v>
+      </c>
+      <c r="T2" s="18">
+        <f t="shared" si="0"/>
+        <v>741000</v>
+      </c>
+      <c r="U2" s="18">
+        <f t="shared" si="0"/>
+        <v>741000</v>
+      </c>
+      <c r="V2" s="18">
+        <f t="shared" si="0"/>
+        <v>741000</v>
+      </c>
+      <c r="W2" s="18">
+        <f t="shared" si="0"/>
+        <v>741000</v>
+      </c>
+      <c r="X2" s="18">
+        <f t="shared" si="0"/>
+        <v>741000</v>
+      </c>
+      <c r="Y2" s="18">
+        <f t="shared" si="0"/>
+        <v>741000</v>
+      </c>
+      <c r="Z2" s="19">
+        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$20</f>
+        <v>741000</v>
+      </c>
+      <c r="AA2" s="19">
+        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$20</f>
+        <v>741000</v>
+      </c>
+      <c r="AB2" s="19">
+        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$20</f>
+        <v>741000</v>
+      </c>
+      <c r="AC2" s="19">
+        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$20</f>
+        <v>741000</v>
+      </c>
+      <c r="AD2" s="19">
+        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$20</f>
+        <v>741000</v>
+      </c>
+      <c r="AE2" s="19">
+        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$20</f>
+        <v>741000</v>
+      </c>
+      <c r="AF2" s="19">
+        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$20</f>
+        <v>741000</v>
+      </c>
+      <c r="AG2" s="19">
+        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$20</f>
+        <v>741000</v>
+      </c>
+      <c r="AH2" s="19">
+        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$20</f>
+        <v>741000</v>
+      </c>
+      <c r="AI2" s="19">
+        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$20</f>
+        <v>741000</v>
+      </c>
+      <c r="AJ2" s="19">
+        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$20</f>
+        <v>741000</v>
+      </c>
+      <c r="AK2" s="19">
+        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$20</f>
+        <v>741000</v>
+      </c>
+      <c r="AL2" s="19">
+        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$20</f>
+        <v>741000</v>
+      </c>
+      <c r="AM2" s="19">
+        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$20</f>
+        <v>741000</v>
+      </c>
+      <c r="AN2" s="19">
+        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$20</f>
+        <v>741000</v>
+      </c>
+      <c r="AO2" s="19">
+        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$20</f>
+        <v>741000</v>
+      </c>
+      <c r="AP2" s="19">
+        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$20</f>
+        <v>741000</v>
+      </c>
+      <c r="AQ2" s="19">
+        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$20</f>
+        <v>741000</v>
+      </c>
+      <c r="AR2" s="19">
+        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$20</f>
+        <v>741000</v>
+      </c>
+      <c r="AS2" s="19">
+        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$20</f>
+        <v>741000</v>
+      </c>
+      <c r="AT2" s="19">
+        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$20</f>
+        <v>741000</v>
+      </c>
+      <c r="AU2" s="19">
+        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$20</f>
+        <v>741000</v>
+      </c>
+      <c r="AV2" s="19">
+        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$20</f>
+        <v>741000</v>
+      </c>
+      <c r="AW2" s="19">
+        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$20</f>
+        <v>741000</v>
+      </c>
+      <c r="AX2" s="19">
+        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$20</f>
+        <v>741000</v>
+      </c>
+      <c r="AY2" s="19">
+        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$20</f>
+        <v>741000</v>
+      </c>
+      <c r="AZ2" s="19">
+        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$20</f>
+        <v>741000</v>
+      </c>
+      <c r="BA2" s="19">
+        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$20</f>
+        <v>741000</v>
+      </c>
+      <c r="BB2" s="19">
+        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$20</f>
+        <v>741000</v>
+      </c>
+      <c r="BC2" s="19">
+        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$20</f>
+        <v>741000</v>
+      </c>
+      <c r="BD2" s="19">
+        <f>'Calculations &amp; Conversions'!$C$12/'Calculations &amp; Conversions'!$E$20</f>
+        <v>741000</v>
       </c>
     </row>
     <row r="3" spans="1:56">
       <c r="A3" t="s">
-        <v>26</v>
+        <v>57</v>
       </c>
       <c r="B3" s="3">
-        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$10</f>
-        <v>345800</v>
+        <f>'Calculations &amp; Conversions'!$C13/'Calculations &amp; Conversions'!$E$19</f>
+        <v>518700</v>
       </c>
       <c r="C3" s="3">
-        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$10</f>
-        <v>345800</v>
+        <f>'Calculations &amp; Conversions'!$C13/'Calculations &amp; Conversions'!$E$19</f>
+        <v>518700</v>
       </c>
       <c r="D3" s="3">
-        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$10</f>
-        <v>345800</v>
+        <f>'Calculations &amp; Conversions'!$C13/'Calculations &amp; Conversions'!$E$19</f>
+        <v>518700</v>
       </c>
       <c r="E3" s="3">
-        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$10</f>
-        <v>345800</v>
+        <f>'Calculations &amp; Conversions'!$C13/'Calculations &amp; Conversions'!$E$19</f>
+        <v>518700</v>
       </c>
       <c r="F3" s="3">
-        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$10</f>
-        <v>345800</v>
+        <f>'Calculations &amp; Conversions'!$C13/'Calculations &amp; Conversions'!$E$19</f>
+        <v>518700</v>
       </c>
       <c r="G3" s="3">
-        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$10</f>
-        <v>345800</v>
+        <f>'Calculations &amp; Conversions'!$C13/'Calculations &amp; Conversions'!$E$19</f>
+        <v>518700</v>
       </c>
       <c r="H3" s="3">
-        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$10</f>
-        <v>345800</v>
+        <f>'Calculations &amp; Conversions'!$C13/'Calculations &amp; Conversions'!$E$19</f>
+        <v>518700</v>
       </c>
       <c r="I3" s="3">
-        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$10</f>
-        <v>345800</v>
+        <f>'Calculations &amp; Conversions'!$C13/'Calculations &amp; Conversions'!$E$19</f>
+        <v>518700</v>
       </c>
       <c r="J3" s="3">
-        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$10</f>
-        <v>345800</v>
+        <f>'Calculations &amp; Conversions'!$C13/'Calculations &amp; Conversions'!$E$19</f>
+        <v>518700</v>
       </c>
       <c r="K3" s="3">
-        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$10</f>
-        <v>345800</v>
+        <f>'Calculations &amp; Conversions'!$C13/'Calculations &amp; Conversions'!$E$19</f>
+        <v>518700</v>
       </c>
       <c r="L3" s="3">
-        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$10</f>
-        <v>345800</v>
+        <f>'Calculations &amp; Conversions'!$C13/'Calculations &amp; Conversions'!$E$19</f>
+        <v>518700</v>
       </c>
       <c r="M3" s="3">
-        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$10</f>
-        <v>345800</v>
+        <f>'Calculations &amp; Conversions'!$C13/'Calculations &amp; Conversions'!$E$19</f>
+        <v>518700</v>
       </c>
       <c r="N3" s="3">
-        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$10</f>
-        <v>345800</v>
+        <f>'Calculations &amp; Conversions'!$C13/'Calculations &amp; Conversions'!$E$19</f>
+        <v>518700</v>
       </c>
       <c r="O3" s="3">
-        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$10</f>
-        <v>345800</v>
+        <f>'Calculations &amp; Conversions'!$C13/'Calculations &amp; Conversions'!$E$19</f>
+        <v>518700</v>
       </c>
       <c r="P3" s="3">
-        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$10</f>
-        <v>345800</v>
-      </c>
-      <c r="Q3" s="3">
-        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$10</f>
-        <v>345800</v>
-      </c>
-      <c r="R3" s="3">
-        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$10</f>
-        <v>345800</v>
-      </c>
-      <c r="S3" s="3">
-        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$10</f>
-        <v>345800</v>
-      </c>
-      <c r="T3" s="3">
-        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$10</f>
-        <v>345800</v>
-      </c>
-      <c r="U3" s="3">
-        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$10</f>
-        <v>345800</v>
-      </c>
-      <c r="V3" s="3">
-        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$10</f>
-        <v>345800</v>
-      </c>
-      <c r="W3" s="3">
-        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$10</f>
-        <v>345800</v>
-      </c>
-      <c r="X3" s="3">
-        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$10</f>
-        <v>345800</v>
-      </c>
-      <c r="Y3" s="3">
-        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$10</f>
-        <v>345800</v>
-      </c>
-      <c r="Z3" s="3">
-        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$10</f>
-        <v>345800</v>
-      </c>
-      <c r="AA3" s="3">
-        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$10</f>
-        <v>345800</v>
-      </c>
-      <c r="AB3" s="3">
-        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$10</f>
-        <v>345800</v>
-      </c>
-      <c r="AC3" s="3">
-        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$10</f>
-        <v>345800</v>
-      </c>
-      <c r="AD3" s="3">
-        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$10</f>
-        <v>345800</v>
-      </c>
-      <c r="AE3" s="3">
-        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$10</f>
-        <v>345800</v>
-      </c>
-      <c r="AF3" s="3">
-        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$10</f>
-        <v>345800</v>
-      </c>
-      <c r="AG3" s="3">
-        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$10</f>
-        <v>345800</v>
-      </c>
-      <c r="AH3" s="3">
-        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$10</f>
-        <v>345800</v>
-      </c>
-      <c r="AI3" s="3">
-        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$10</f>
-        <v>345800</v>
-      </c>
-      <c r="AJ3" s="3">
-        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$10</f>
-        <v>345800</v>
-      </c>
-      <c r="AK3" s="3">
-        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$10</f>
-        <v>345800</v>
-      </c>
-      <c r="AL3" s="3">
-        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$10</f>
-        <v>345800</v>
-      </c>
-      <c r="AM3" s="3">
-        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$10</f>
-        <v>345800</v>
-      </c>
-      <c r="AN3" s="3">
-        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$10</f>
-        <v>345800</v>
-      </c>
-      <c r="AO3" s="3">
-        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$10</f>
-        <v>345800</v>
-      </c>
-      <c r="AP3" s="3">
-        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$10</f>
-        <v>345800</v>
-      </c>
-      <c r="AQ3" s="3">
-        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$10</f>
-        <v>345800</v>
-      </c>
-      <c r="AR3" s="3">
-        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$10</f>
-        <v>345800</v>
-      </c>
-      <c r="AS3" s="3">
-        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$10</f>
-        <v>345800</v>
-      </c>
-      <c r="AT3" s="3">
-        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$10</f>
-        <v>345800</v>
-      </c>
-      <c r="AU3" s="3">
-        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$10</f>
-        <v>345800</v>
-      </c>
-      <c r="AV3" s="3">
-        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$10</f>
-        <v>345800</v>
-      </c>
-      <c r="AW3" s="3">
-        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$10</f>
-        <v>345800</v>
-      </c>
-      <c r="AX3" s="3">
-        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$10</f>
-        <v>345800</v>
-      </c>
-      <c r="AY3" s="3">
-        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$10</f>
-        <v>345800</v>
-      </c>
-      <c r="AZ3" s="3">
-        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$10</f>
-        <v>345800</v>
-      </c>
-      <c r="BA3" s="3">
-        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$10</f>
-        <v>345800</v>
-      </c>
-      <c r="BB3" s="3">
-        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$10</f>
-        <v>345800</v>
-      </c>
-      <c r="BC3" s="3">
-        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$10</f>
-        <v>345800</v>
-      </c>
-      <c r="BD3" s="3">
-        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$10</f>
-        <v>345800</v>
+        <f>'Calculations &amp; Conversions'!$C13/'Calculations &amp; Conversions'!$E$19</f>
+        <v>518700</v>
+      </c>
+      <c r="Q3" s="18">
+        <f>(Z3-P3)/(Z$1-P$1)*(Q$1-$P$1)+$P3</f>
+        <v>518700</v>
+      </c>
+      <c r="R3" s="18">
+        <f t="shared" ref="R3:R7" si="1">(AA3-Q3)/(AA$1-Q$1)*(R$1-$P$1)+$P3</f>
+        <v>518700</v>
+      </c>
+      <c r="S3" s="18">
+        <f t="shared" ref="S3:S7" si="2">(AB3-R3)/(AB$1-R$1)*(S$1-$P$1)+$P3</f>
+        <v>518700</v>
+      </c>
+      <c r="T3" s="18">
+        <f t="shared" ref="T3:T7" si="3">(AC3-S3)/(AC$1-S$1)*(T$1-$P$1)+$P3</f>
+        <v>518700</v>
+      </c>
+      <c r="U3" s="18">
+        <f t="shared" ref="U3:U7" si="4">(AD3-T3)/(AD$1-T$1)*(U$1-$P$1)+$P3</f>
+        <v>518700</v>
+      </c>
+      <c r="V3" s="18">
+        <f t="shared" ref="V3:V7" si="5">(AE3-U3)/(AE$1-U$1)*(V$1-$P$1)+$P3</f>
+        <v>518700</v>
+      </c>
+      <c r="W3" s="18">
+        <f t="shared" ref="W3:W7" si="6">(AF3-V3)/(AF$1-V$1)*(W$1-$P$1)+$P3</f>
+        <v>518700</v>
+      </c>
+      <c r="X3" s="18">
+        <f t="shared" ref="X3:X7" si="7">(AG3-W3)/(AG$1-W$1)*(X$1-$P$1)+$P3</f>
+        <v>518700</v>
+      </c>
+      <c r="Y3" s="18">
+        <f t="shared" ref="Y3:Y7" si="8">(AH3-X3)/(AH$1-X$1)*(Y$1-$P$1)+$P3</f>
+        <v>518700</v>
+      </c>
+      <c r="Z3" s="19">
+        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$20</f>
+        <v>518700</v>
+      </c>
+      <c r="AA3" s="19">
+        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$20</f>
+        <v>518700</v>
+      </c>
+      <c r="AB3" s="19">
+        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$20</f>
+        <v>518700</v>
+      </c>
+      <c r="AC3" s="19">
+        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$20</f>
+        <v>518700</v>
+      </c>
+      <c r="AD3" s="19">
+        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$20</f>
+        <v>518700</v>
+      </c>
+      <c r="AE3" s="19">
+        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$20</f>
+        <v>518700</v>
+      </c>
+      <c r="AF3" s="19">
+        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$20</f>
+        <v>518700</v>
+      </c>
+      <c r="AG3" s="19">
+        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$20</f>
+        <v>518700</v>
+      </c>
+      <c r="AH3" s="19">
+        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$20</f>
+        <v>518700</v>
+      </c>
+      <c r="AI3" s="19">
+        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$20</f>
+        <v>518700</v>
+      </c>
+      <c r="AJ3" s="19">
+        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$20</f>
+        <v>518700</v>
+      </c>
+      <c r="AK3" s="19">
+        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$20</f>
+        <v>518700</v>
+      </c>
+      <c r="AL3" s="19">
+        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$20</f>
+        <v>518700</v>
+      </c>
+      <c r="AM3" s="19">
+        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$20</f>
+        <v>518700</v>
+      </c>
+      <c r="AN3" s="19">
+        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$20</f>
+        <v>518700</v>
+      </c>
+      <c r="AO3" s="19">
+        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$20</f>
+        <v>518700</v>
+      </c>
+      <c r="AP3" s="19">
+        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$20</f>
+        <v>518700</v>
+      </c>
+      <c r="AQ3" s="19">
+        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$20</f>
+        <v>518700</v>
+      </c>
+      <c r="AR3" s="19">
+        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$20</f>
+        <v>518700</v>
+      </c>
+      <c r="AS3" s="19">
+        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$20</f>
+        <v>518700</v>
+      </c>
+      <c r="AT3" s="19">
+        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$20</f>
+        <v>518700</v>
+      </c>
+      <c r="AU3" s="19">
+        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$20</f>
+        <v>518700</v>
+      </c>
+      <c r="AV3" s="19">
+        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$20</f>
+        <v>518700</v>
+      </c>
+      <c r="AW3" s="19">
+        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$20</f>
+        <v>518700</v>
+      </c>
+      <c r="AX3" s="19">
+        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$20</f>
+        <v>518700</v>
+      </c>
+      <c r="AY3" s="19">
+        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$20</f>
+        <v>518700</v>
+      </c>
+      <c r="AZ3" s="19">
+        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$20</f>
+        <v>518700</v>
+      </c>
+      <c r="BA3" s="19">
+        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$20</f>
+        <v>518700</v>
+      </c>
+      <c r="BB3" s="19">
+        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$20</f>
+        <v>518700</v>
+      </c>
+      <c r="BC3" s="19">
+        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$20</f>
+        <v>518700</v>
+      </c>
+      <c r="BD3" s="19">
+        <f>'Calculations &amp; Conversions'!$C$13/'Calculations &amp; Conversions'!$E$20</f>
+        <v>518700</v>
       </c>
     </row>
     <row r="4" spans="1:56">
       <c r="A4" t="s">
-        <v>27</v>
+        <v>58</v>
       </c>
       <c r="B4" s="3">
-        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$10</f>
-        <v>1696066.6666666667</v>
+        <f>'Calculations &amp; Conversions'!$C14/'Calculations &amp; Conversions'!$E$19</f>
+        <v>2309450</v>
       </c>
       <c r="C4" s="3">
-        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$10</f>
-        <v>1696066.6666666667</v>
+        <f>'Calculations &amp; Conversions'!$C14/'Calculations &amp; Conversions'!$E$19</f>
+        <v>2309450</v>
       </c>
       <c r="D4" s="3">
-        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$10</f>
-        <v>1696066.6666666667</v>
+        <f>'Calculations &amp; Conversions'!$C14/'Calculations &amp; Conversions'!$E$19</f>
+        <v>2309450</v>
       </c>
       <c r="E4" s="3">
-        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$10</f>
-        <v>1696066.6666666667</v>
+        <f>'Calculations &amp; Conversions'!$C14/'Calculations &amp; Conversions'!$E$19</f>
+        <v>2309450</v>
       </c>
       <c r="F4" s="3">
-        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$10</f>
-        <v>1696066.6666666667</v>
+        <f>'Calculations &amp; Conversions'!$C14/'Calculations &amp; Conversions'!$E$19</f>
+        <v>2309450</v>
       </c>
       <c r="G4" s="3">
-        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$10</f>
-        <v>1696066.6666666667</v>
+        <f>'Calculations &amp; Conversions'!$C14/'Calculations &amp; Conversions'!$E$19</f>
+        <v>2309450</v>
       </c>
       <c r="H4" s="3">
-        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$10</f>
-        <v>1696066.6666666667</v>
+        <f>'Calculations &amp; Conversions'!$C14/'Calculations &amp; Conversions'!$E$19</f>
+        <v>2309450</v>
       </c>
       <c r="I4" s="3">
-        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$10</f>
-        <v>1696066.6666666667</v>
+        <f>'Calculations &amp; Conversions'!$C14/'Calculations &amp; Conversions'!$E$19</f>
+        <v>2309450</v>
       </c>
       <c r="J4" s="3">
-        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$10</f>
-        <v>1696066.6666666667</v>
+        <f>'Calculations &amp; Conversions'!$C14/'Calculations &amp; Conversions'!$E$19</f>
+        <v>2309450</v>
       </c>
       <c r="K4" s="3">
-        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$10</f>
-        <v>1696066.6666666667</v>
+        <f>'Calculations &amp; Conversions'!$C14/'Calculations &amp; Conversions'!$E$19</f>
+        <v>2309450</v>
       </c>
       <c r="L4" s="3">
-        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$10</f>
-        <v>1696066.6666666667</v>
+        <f>'Calculations &amp; Conversions'!$C14/'Calculations &amp; Conversions'!$E$19</f>
+        <v>2309450</v>
       </c>
       <c r="M4" s="3">
-        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$10</f>
-        <v>1696066.6666666667</v>
+        <f>'Calculations &amp; Conversions'!$C14/'Calculations &amp; Conversions'!$E$19</f>
+        <v>2309450</v>
       </c>
       <c r="N4" s="3">
-        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$10</f>
-        <v>1696066.6666666667</v>
+        <f>'Calculations &amp; Conversions'!$C14/'Calculations &amp; Conversions'!$E$19</f>
+        <v>2309450</v>
       </c>
       <c r="O4" s="3">
-        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$10</f>
-        <v>1696066.6666666667</v>
+        <f>'Calculations &amp; Conversions'!$C14/'Calculations &amp; Conversions'!$E$19</f>
+        <v>2309450</v>
       </c>
       <c r="P4" s="3">
-        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$10</f>
-        <v>1696066.6666666667</v>
-      </c>
-      <c r="Q4" s="3">
-        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$10</f>
-        <v>1696066.6666666667</v>
-      </c>
-      <c r="R4" s="3">
-        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$10</f>
-        <v>1696066.6666666667</v>
-      </c>
-      <c r="S4" s="3">
-        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$10</f>
-        <v>1696066.6666666667</v>
-      </c>
-      <c r="T4" s="3">
-        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$10</f>
-        <v>1696066.6666666667</v>
-      </c>
-      <c r="U4" s="3">
-        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$10</f>
-        <v>1696066.6666666667</v>
-      </c>
-      <c r="V4" s="3">
-        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$10</f>
-        <v>1696066.6666666667</v>
-      </c>
-      <c r="W4" s="3">
-        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$10</f>
-        <v>1696066.6666666667</v>
-      </c>
-      <c r="X4" s="3">
-        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$10</f>
-        <v>1696066.6666666667</v>
-      </c>
-      <c r="Y4" s="3">
-        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$10</f>
-        <v>1696066.6666666667</v>
-      </c>
-      <c r="Z4" s="3">
-        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$10</f>
-        <v>1696066.6666666667</v>
-      </c>
-      <c r="AA4" s="3">
-        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$10</f>
-        <v>1696066.6666666667</v>
-      </c>
-      <c r="AB4" s="3">
-        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$10</f>
-        <v>1696066.6666666667</v>
-      </c>
-      <c r="AC4" s="3">
-        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$10</f>
-        <v>1696066.6666666667</v>
-      </c>
-      <c r="AD4" s="3">
-        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$10</f>
-        <v>1696066.6666666667</v>
-      </c>
-      <c r="AE4" s="3">
-        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$10</f>
-        <v>1696066.6666666667</v>
-      </c>
-      <c r="AF4" s="3">
-        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$10</f>
-        <v>1696066.6666666667</v>
-      </c>
-      <c r="AG4" s="3">
-        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$10</f>
-        <v>1696066.6666666667</v>
-      </c>
-      <c r="AH4" s="3">
-        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$10</f>
-        <v>1696066.6666666667</v>
-      </c>
-      <c r="AI4" s="3">
-        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$10</f>
-        <v>1696066.6666666667</v>
-      </c>
-      <c r="AJ4" s="3">
-        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$10</f>
-        <v>1696066.6666666667</v>
-      </c>
-      <c r="AK4" s="3">
-        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$10</f>
-        <v>1696066.6666666667</v>
-      </c>
-      <c r="AL4" s="3">
-        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$10</f>
-        <v>1696066.6666666667</v>
-      </c>
-      <c r="AM4" s="3">
-        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$10</f>
-        <v>1696066.6666666667</v>
-      </c>
-      <c r="AN4" s="3">
-        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$10</f>
-        <v>1696066.6666666667</v>
-      </c>
-      <c r="AO4" s="3">
-        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$10</f>
-        <v>1696066.6666666667</v>
-      </c>
-      <c r="AP4" s="3">
-        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$10</f>
-        <v>1696066.6666666667</v>
-      </c>
-      <c r="AQ4" s="3">
-        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$10</f>
-        <v>1696066.6666666667</v>
-      </c>
-      <c r="AR4" s="3">
-        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$10</f>
-        <v>1696066.6666666667</v>
-      </c>
-      <c r="AS4" s="3">
-        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$10</f>
-        <v>1696066.6666666667</v>
-      </c>
-      <c r="AT4" s="3">
-        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$10</f>
-        <v>1696066.6666666667</v>
-      </c>
-      <c r="AU4" s="3">
-        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$10</f>
-        <v>1696066.6666666667</v>
-      </c>
-      <c r="AV4" s="3">
-        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$10</f>
-        <v>1696066.6666666667</v>
-      </c>
-      <c r="AW4" s="3">
-        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$10</f>
-        <v>1696066.6666666667</v>
-      </c>
-      <c r="AX4" s="3">
-        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$10</f>
-        <v>1696066.6666666667</v>
-      </c>
-      <c r="AY4" s="3">
-        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$10</f>
-        <v>1696066.6666666667</v>
-      </c>
-      <c r="AZ4" s="3">
-        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$10</f>
-        <v>1696066.6666666667</v>
-      </c>
-      <c r="BA4" s="3">
-        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$10</f>
-        <v>1696066.6666666667</v>
-      </c>
-      <c r="BB4" s="3">
-        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$10</f>
-        <v>1696066.6666666667</v>
-      </c>
-      <c r="BC4" s="3">
-        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$10</f>
-        <v>1696066.6666666667</v>
-      </c>
-      <c r="BD4" s="3">
-        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$10</f>
-        <v>1696066.6666666667</v>
+        <f>'Calculations &amp; Conversions'!$C14/'Calculations &amp; Conversions'!$E$19</f>
+        <v>2309450</v>
+      </c>
+      <c r="Q4" s="18">
+        <f t="shared" ref="Q3:Q7" si="9">(Z4-P4)/(Z$1-P$1)*(Q$1-$P$1)+$P4</f>
+        <v>2332915</v>
+      </c>
+      <c r="R4" s="18">
+        <f t="shared" si="1"/>
+        <v>2351687</v>
+      </c>
+      <c r="S4" s="18">
+        <f t="shared" si="2"/>
+        <v>2367173.9</v>
+      </c>
+      <c r="T4" s="18">
+        <f t="shared" si="3"/>
+        <v>2380220.44</v>
+      </c>
+      <c r="U4" s="18">
+        <f t="shared" si="4"/>
+        <v>2391389.7800000003</v>
+      </c>
+      <c r="V4" s="18">
+        <f t="shared" si="5"/>
+        <v>2401076.1319999998</v>
+      </c>
+      <c r="W4" s="18">
+        <f t="shared" si="6"/>
+        <v>2409566.7076000003</v>
+      </c>
+      <c r="X4" s="18">
+        <f t="shared" si="7"/>
+        <v>2417076.6339199999</v>
+      </c>
+      <c r="Y4" s="18">
+        <f t="shared" si="8"/>
+        <v>2423771.029472</v>
+      </c>
+      <c r="Z4" s="19">
+        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$20</f>
+        <v>2544100</v>
+      </c>
+      <c r="AA4" s="19">
+        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$20</f>
+        <v>2544100</v>
+      </c>
+      <c r="AB4" s="19">
+        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$20</f>
+        <v>2544100</v>
+      </c>
+      <c r="AC4" s="19">
+        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$20</f>
+        <v>2544100</v>
+      </c>
+      <c r="AD4" s="19">
+        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$20</f>
+        <v>2544100</v>
+      </c>
+      <c r="AE4" s="19">
+        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$20</f>
+        <v>2544100</v>
+      </c>
+      <c r="AF4" s="19">
+        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$20</f>
+        <v>2544100</v>
+      </c>
+      <c r="AG4" s="19">
+        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$20</f>
+        <v>2544100</v>
+      </c>
+      <c r="AH4" s="19">
+        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$20</f>
+        <v>2544100</v>
+      </c>
+      <c r="AI4" s="19">
+        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$20</f>
+        <v>2544100</v>
+      </c>
+      <c r="AJ4" s="19">
+        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$20</f>
+        <v>2544100</v>
+      </c>
+      <c r="AK4" s="19">
+        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$20</f>
+        <v>2544100</v>
+      </c>
+      <c r="AL4" s="19">
+        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$20</f>
+        <v>2544100</v>
+      </c>
+      <c r="AM4" s="19">
+        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$20</f>
+        <v>2544100</v>
+      </c>
+      <c r="AN4" s="19">
+        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$20</f>
+        <v>2544100</v>
+      </c>
+      <c r="AO4" s="19">
+        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$20</f>
+        <v>2544100</v>
+      </c>
+      <c r="AP4" s="19">
+        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$20</f>
+        <v>2544100</v>
+      </c>
+      <c r="AQ4" s="19">
+        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$20</f>
+        <v>2544100</v>
+      </c>
+      <c r="AR4" s="19">
+        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$20</f>
+        <v>2544100</v>
+      </c>
+      <c r="AS4" s="19">
+        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$20</f>
+        <v>2544100</v>
+      </c>
+      <c r="AT4" s="19">
+        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$20</f>
+        <v>2544100</v>
+      </c>
+      <c r="AU4" s="19">
+        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$20</f>
+        <v>2544100</v>
+      </c>
+      <c r="AV4" s="19">
+        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$20</f>
+        <v>2544100</v>
+      </c>
+      <c r="AW4" s="19">
+        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$20</f>
+        <v>2544100</v>
+      </c>
+      <c r="AX4" s="19">
+        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$20</f>
+        <v>2544100</v>
+      </c>
+      <c r="AY4" s="19">
+        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$20</f>
+        <v>2544100</v>
+      </c>
+      <c r="AZ4" s="19">
+        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$20</f>
+        <v>2544100</v>
+      </c>
+      <c r="BA4" s="19">
+        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$20</f>
+        <v>2544100</v>
+      </c>
+      <c r="BB4" s="19">
+        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$20</f>
+        <v>2544100</v>
+      </c>
+      <c r="BC4" s="19">
+        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$20</f>
+        <v>2544100</v>
+      </c>
+      <c r="BD4" s="19">
+        <f>('Calculations &amp; Conversions'!$C$14+'Calculations &amp; Conversions'!$C$15)/'Calculations &amp; Conversions'!$E$20</f>
+        <v>2544100</v>
       </c>
     </row>
     <row r="5" spans="1:56">
       <c r="A5" t="s">
-        <v>28</v>
+        <v>59</v>
       </c>
       <c r="B5" s="3">
         <v>0</v>
@@ -1853,31 +2527,40 @@
       <c r="P5" s="3">
         <v>0</v>
       </c>
-      <c r="Q5" s="3">
-        <v>0</v>
-      </c>
-      <c r="R5" s="3">
-        <v>0</v>
-      </c>
-      <c r="S5" s="3">
-        <v>0</v>
-      </c>
-      <c r="T5" s="3">
-        <v>0</v>
-      </c>
-      <c r="U5" s="3">
-        <v>0</v>
-      </c>
-      <c r="V5" s="3">
-        <v>0</v>
-      </c>
-      <c r="W5" s="3">
-        <v>0</v>
-      </c>
-      <c r="X5" s="3">
-        <v>0</v>
-      </c>
-      <c r="Y5" s="3">
+      <c r="Q5" s="18">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="R5" s="18">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="S5" s="18">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="T5" s="18">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U5" s="18">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V5" s="18">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="W5" s="18">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="X5" s="18">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="Y5" s="18">
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="Z5" s="3">
@@ -1976,7 +2659,7 @@
     </row>
     <row r="6" spans="1:56">
       <c r="A6" t="s">
-        <v>29</v>
+        <v>60</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -2023,31 +2706,40 @@
       <c r="P6">
         <v>0</v>
       </c>
-      <c r="Q6">
-        <v>0</v>
-      </c>
-      <c r="R6">
-        <v>0</v>
-      </c>
-      <c r="S6">
-        <v>0</v>
-      </c>
-      <c r="T6">
-        <v>0</v>
-      </c>
-      <c r="U6">
-        <v>0</v>
-      </c>
-      <c r="V6">
-        <v>0</v>
-      </c>
-      <c r="W6">
-        <v>0</v>
-      </c>
-      <c r="X6">
-        <v>0</v>
-      </c>
-      <c r="Y6">
+      <c r="Q6" s="18">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="R6" s="18">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="S6" s="18">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="T6" s="18">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U6" s="18">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V6" s="18">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="W6" s="18">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="X6" s="18">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="Y6" s="18">
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="Z6">
@@ -2146,7 +2838,7 @@
     </row>
     <row r="7" spans="1:56">
       <c r="A7" t="s">
-        <v>30</v>
+        <v>61</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -2193,31 +2885,40 @@
       <c r="P7">
         <v>0</v>
       </c>
-      <c r="Q7">
-        <v>0</v>
-      </c>
-      <c r="R7">
-        <v>0</v>
-      </c>
-      <c r="S7">
-        <v>0</v>
-      </c>
-      <c r="T7">
-        <v>0</v>
-      </c>
-      <c r="U7">
-        <v>0</v>
-      </c>
-      <c r="V7">
-        <v>0</v>
-      </c>
-      <c r="W7">
-        <v>0</v>
-      </c>
-      <c r="X7">
-        <v>0</v>
-      </c>
-      <c r="Y7">
+      <c r="Q7" s="18">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="R7" s="18">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="S7" s="18">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="T7" s="18">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U7" s="18">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V7" s="18">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="W7" s="18">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="X7" s="18">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="Y7" s="18">
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="Z7">
@@ -2323,14 +3024,17 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101009A9DAB439B36DB4795F39C4E722C7BC4" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="44674c89fa9bc5e97a878a6680c46188">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="79748b23-d81a-423e-9112-21109dc864e6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="447839a363ea5a12024b5bf1ab53ed90" ns2:_="">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101009A9DAB439B36DB4795F39C4E722C7BC4" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="6b365794f824c3a5fb2e977be4d8f3b3">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="79748b23-d81a-423e-9112-21109dc864e6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="e910879461a45d0cdddc64f187ce3652" ns2:_="">
     <xsd:import namespace="79748b23-d81a-423e-9112-21109dc864e6"/>
     <xsd:element name="properties">
       <xsd:complexType>
@@ -2473,22 +3177,19 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C1A869E2-791B-41A0-B65B-6011022F31CC}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0085AE3C-E105-4F11-98DA-4EE89E9D85CC}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7CE26BC1-C84C-4C3F-990C-52F7BA333174}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ED40BE3F-2539-4D6A-AD05-872209C36F4A}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0085AE3C-E105-4F11-98DA-4EE89E9D85CC}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C1A869E2-791B-41A0-B65B-6011022F31CC}"/>
 </file>
</xml_diff>